<commit_message>
Klart för Power BI
</commit_message>
<xml_diff>
--- a/Projektplan.xlsx
+++ b/Projektplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michael.brostrom\Documents\GitHub\statistik-freshdesk-linear\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1857891-4BB2-4865-BDB8-30BCE2D38E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8584E54-1A62-41CB-A4A9-EB8198036C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-46188" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{6423C684-42E7-44D6-BC0D-A51FB6EB8C31}"/>
+    <workbookView xWindow="-46188" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{6423C684-42E7-44D6-BC0D-A51FB6EB8C31}"/>
   </bookViews>
   <sheets>
     <sheet name="Översikt" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Star Schema" sheetId="7" r:id="rId5"/>
     <sheet name="Loggbok" sheetId="4" r:id="rId6"/>
     <sheet name="KPI-vyer" sheetId="8" r:id="rId7"/>
+    <sheet name="Uppgifter (old)" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -46,26 +47,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="317">
   <si>
     <t>Steg 2</t>
   </si>
   <si>
     <t xml:space="preserve">Steg 1 </t>
-  </si>
-  <si>
-    <r>
-      <t>Bronze:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Kombinera Linear + Freshdesk till en append‑only bronze_master; spara metadata och loggar.</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">Steg 3 </t>
@@ -1044,12 +1031,89 @@
   <si>
     <t>To date</t>
   </si>
+  <si>
+    <t>Reset</t>
+  </si>
+  <si>
+    <t>Börja om från början med nya förutsättningar</t>
+  </si>
+  <si>
+    <t>Script, storage, logic, PBI</t>
+  </si>
+  <si>
+    <r>
+      <t>Bronze:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Kombinera Linear + Freshdesk till append‑only bronze_master-filer; spara metadata och loggar.</t>
+    </r>
+  </si>
+  <si>
+    <t>Att göra efter sample visuals-experimentet</t>
+  </si>
+  <si>
+    <t>Gå igenom fält och bestäm vilka som är viktiga</t>
+  </si>
+  <si>
+    <t>30 dagar fönster på Freshdesk räcker</t>
+  </si>
+  <si>
+    <t>Ny backfill med raw JSON från Linear och Freshdesk</t>
+  </si>
+  <si>
+    <t>Skapa automatisering</t>
+  </si>
+  <si>
+    <t>Github repo access</t>
+  </si>
+  <si>
+    <t>Github actions klara och testade. Nattkörning görs nu framöver</t>
+  </si>
+  <si>
+    <t>Ta in Linear och Freshdesk json till ett append‑only bronze_lager</t>
+  </si>
+  <si>
+    <t>Json-filer i Github repo</t>
+  </si>
+  <si>
+    <t>SQL Server</t>
+  </si>
+  <si>
+    <t>Migrera hela projektet till nätverksserver istf localhost</t>
+  </si>
+  <si>
+    <t>INTSQLSERVER01/InternalStatistics</t>
+  </si>
+  <si>
+    <t>/credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SQL Server Authentication-login i /credentials </t>
+  </si>
+  <si>
+    <t>Städat bort mycket irrelevant från Freshdesk och en del från Linear.</t>
+  </si>
+  <si>
+    <t>Generera DimDate för 2025–2035 med daglig granularitet och diverse "smarta" kolumner för hanteringen.</t>
+  </si>
+  <si>
+    <t>Daglig granularitet. Helgdagar och annat inlagt för att kunna normalisera volymer över veckor.</t>
+  </si>
+  <si>
+    <t>Skapa vyer i Gold-lagret så att PBI via dessa kommer åt data från Silverlagret (som blir det sista som uppdateras från rådata - via bronze).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1106,6 +1170,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1139,7 +1210,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1189,12 +1260,84 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="43">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1482,67 +1625,89 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}" name="Table3" displayName="Table3" ref="A1:J17" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:J17" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J17">
-    <sortCondition ref="A5:A17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}" name="Table3" displayName="Table3" ref="A3:J20" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+  <autoFilter ref="A3:J20" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:J20">
+    <sortCondition ref="A4:A20"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{621EA786-D68B-4811-8816-275E67518CF7}" name="ID" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{F932A01A-5B0D-40FB-AEE9-1CED13B12D94}" name="Uppgift" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{ACF35F41-358C-4CB0-8D97-0779A9D2BAE9}" name="Beskrivning" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{DE3EADD2-F620-4BA4-A481-16B78C3A4973}" name="Start" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{0759F001-4F97-43C5-8D8C-7B3B8459D8CA}" name="Klart" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{D5560EA2-E89A-4EB8-8FED-1B19D1469389}" name="Status" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{DCC81527-DA55-4F19-9225-0DAED3D69C56}" name="Beroenden" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{C1E9D109-8409-480C-A83C-4E5609EB75E1}" name="Leverans" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{65CDC4BE-49D9-4C1B-B16A-361E0A66AF67}" name="Notering" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{D96E1D3D-DDC4-453A-955C-1B6198F24A88}" name="Mapp" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{621EA786-D68B-4811-8816-275E67518CF7}" name="ID" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{F932A01A-5B0D-40FB-AEE9-1CED13B12D94}" name="Uppgift" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{ACF35F41-358C-4CB0-8D97-0779A9D2BAE9}" name="Beskrivning" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{DE3EADD2-F620-4BA4-A481-16B78C3A4973}" name="Start" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{0759F001-4F97-43C5-8D8C-7B3B8459D8CA}" name="Klart" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{D5560EA2-E89A-4EB8-8FED-1B19D1469389}" name="Status" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{DCC81527-DA55-4F19-9225-0DAED3D69C56}" name="Beroenden" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{C1E9D109-8409-480C-A83C-4E5609EB75E1}" name="Leverans" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{65CDC4BE-49D9-4C1B-B16A-361E0A66AF67}" name="Notering" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{D96E1D3D-DDC4-453A-955C-1B6198F24A88}" name="Mapp" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6216B224-B30B-4E9D-92D3-0ADBC32EFFD4}" name="Table7" displayName="Table7" ref="A1:F23" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6216B224-B30B-4E9D-92D3-0ADBC32EFFD4}" name="Table7" displayName="Table7" ref="A1:F23" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:F23" xr:uid="{6216B224-B30B-4E9D-92D3-0ADBC32EFFD4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{7FCF0016-95F2-4F2B-A38F-815761F80B03}" name="Fält" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{AEC41172-11D0-4F04-A0E4-7958638EA435}" name="Datatyp (faktisk)" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{ADB87FC7-FF97-4B0F-A0A0-4C4EE3531B2D}" name="Null‑rate" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{0EBEE600-6B5F-4936-AD1D-717FA1A37244}" name="Cardinalitet" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{58D9AD1A-FD53-4D17-8EE5-FF631CDE3A23}" name="Brons‑normalisering" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{A4CBE5BA-79E3-4F44-B3A4-F2B87C0A6762}" name="Kommentar" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{7FCF0016-95F2-4F2B-A38F-815761F80B03}" name="Fält" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{AEC41172-11D0-4F04-A0E4-7958638EA435}" name="Datatyp (faktisk)" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{ADB87FC7-FF97-4B0F-A0A0-4C4EE3531B2D}" name="Null‑rate" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{0EBEE600-6B5F-4936-AD1D-717FA1A37244}" name="Cardinalitet" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{58D9AD1A-FD53-4D17-8EE5-FF631CDE3A23}" name="Brons‑normalisering" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{A4CBE5BA-79E3-4F44-B3A4-F2B87C0A6762}" name="Kommentar" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0090A6AA-4E64-4D35-895F-4A8F66B9CC17}" name="Table5" displayName="Table5" ref="A1:F40" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0090A6AA-4E64-4D35-895F-4A8F66B9CC17}" name="Table5" displayName="Table5" ref="A1:F40" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
   <autoFilter ref="A1:F40" xr:uid="{0090A6AA-4E64-4D35-895F-4A8F66B9CC17}"/>
   <tableColumns count="6">
-    <tableColumn id="2" xr3:uid="{E6AC1D0F-3726-4BE8-BA46-49840FBE2772}" name="Fält" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{E697331E-6279-430B-A003-C1E4ED054EBA}" name="Korrekt datatyp" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{E9EAA4BD-5BDF-4411-8233-90986A2D9904}" name="Null‑rate" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{888C298A-BDCE-4052-82A8-8332F4F9ADEF}" name="Cardinalitet" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{9346AEEE-448C-4B29-A3E1-DCF2D069DF82}" name="Brons‑normalisering" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{A1697787-E40B-4024-B5FF-F37EAEF1F687}" name="Not" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{E6AC1D0F-3726-4BE8-BA46-49840FBE2772}" name="Fält" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{E697331E-6279-430B-A003-C1E4ED054EBA}" name="Korrekt datatyp" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{E9EAA4BD-5BDF-4411-8233-90986A2D9904}" name="Null‑rate" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{888C298A-BDCE-4052-82A8-8332F4F9ADEF}" name="Cardinalitet" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{9346AEEE-448C-4B29-A3E1-DCF2D069DF82}" name="Brons‑normalisering" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{A1697787-E40B-4024-B5FF-F37EAEF1F687}" name="Not" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{548F0A06-59BD-4EAC-BCA4-2A36F066351C}" name="Table1" displayName="Table1" ref="A1:F9" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:F9" xr:uid="{548F0A06-59BD-4EAC-BCA4-2A36F066351C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{548F0A06-59BD-4EAC-BCA4-2A36F066351C}" name="Table1" displayName="Table1" ref="A1:F10" totalsRowShown="0" headerRowDxfId="15">
+  <autoFilter ref="A1:F10" xr:uid="{548F0A06-59BD-4EAC-BCA4-2A36F066351C}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{AD0E8543-A933-44D5-990C-4A2D887BCB63}" name="Date" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{AD0E8543-A933-44D5-990C-4A2D887BCB63}" name="Date" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{82ACFFA9-0C32-4783-A2DE-E94DB75334AD}" name="Typ"/>
     <tableColumn id="3" xr3:uid="{3B98BD4B-EF41-4872-8E7A-66595C113584}" name="Sammanfattning"/>
     <tableColumn id="4" xr3:uid="{ED260F23-42AE-4AD3-B541-C2EFCA28B066}" name="Detaljer"/>
     <tableColumn id="5" xr3:uid="{EC4FD12B-6929-4080-98FF-5238F7B9AFD5}" name="Att göra"/>
-    <tableColumn id="6" xr3:uid="{58648841-0E5B-4F63-8464-393C743A86A1}" name="Klart" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{58648841-0E5B-4F63-8464-393C743A86A1}" name="Klart" dataDxfId="13"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E3E33F21-3B23-4E2B-807E-F1440673AD2C}" name="Table33" displayName="Table33" ref="A1:J17" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J17" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J17">
+    <sortCondition ref="A5:A17"/>
+  </sortState>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{24EFF8F6-AC33-4FBB-BF8C-47C706E1E2B3}" name="ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{B1C355DA-9E5B-49EA-9267-DB0403B97CD8}" name="Uppgift" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{B469510B-F50B-49AE-BAC0-CAEB00773117}" name="Beskrivning" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{3C0332F4-6929-4C46-8709-36026B81D55E}" name="Start" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{E0864EB4-04EC-491E-9513-B7A38626F65C}" name="Klart" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{B81D0394-E7CF-49DB-898D-DFA6E2C78114}" name="Status" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{25D7BA04-10F0-4DF3-B66A-179388A92C2B}" name="Beroenden" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{7427EEAF-4245-42B1-B742-72A430D54C10}" name="Leverans" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{79563EB4-A3E0-4F2A-AC8B-CF51304768BD}" name="Notering" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{6A71E9D0-42A4-4AA5-AD88-A638A5481E0D}" name="Mapp" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1874,7 +2039,7 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="51" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -1888,7 +2053,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1896,31 +2061,31 @@
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1934,7 +2099,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4FCEBCE-FCD7-407D-A82B-012E341489A8}">
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
@@ -1944,493 +2109,515 @@
     <col min="7" max="7" width="16.5546875" customWidth="1"/>
     <col min="8" max="8" width="19.5546875" customWidth="1"/>
     <col min="9" max="9" width="24.6640625" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
-      <c r="A1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:20" ht="31.2">
+      <c r="A1" s="19" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H3" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="28.8">
+      <c r="A4" s="4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" ht="57.6">
-      <c r="A2" s="4">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" s="6">
-        <v>46170</v>
-      </c>
-      <c r="E2" s="6">
-        <v>46174</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G2" s="5" t="s">
+      <c r="C4" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="D4" s="6">
+        <v>46177</v>
+      </c>
+      <c r="E4" s="6">
+        <v>46177</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:20" ht="43.2">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="D3" s="6">
-        <v>46170</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46174</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-    </row>
-    <row r="4" spans="1:20" ht="57.6">
-      <c r="A4" s="4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="D4" s="6">
-        <v>46174</v>
-      </c>
-      <c r="E4" s="6">
-        <v>46174</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>2</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="J4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="5" spans="1:20" ht="28.8">
       <c r="A5" s="4">
-        <v>4</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="D5" s="11">
-        <v>46174</v>
-      </c>
-      <c r="E5" s="11">
-        <v>46174</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="G5" s="10">
-        <v>3</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="I5" s="10"/>
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D5" s="6">
+        <v>46177</v>
+      </c>
+      <c r="E5" s="6">
+        <v>46177</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>301</v>
+      </c>
       <c r="J5" s="5"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
     </row>
     <row r="6" spans="1:20" ht="43.2">
       <c r="A6" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>19</v>
+        <v>303</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="D6" s="11">
-        <v>46174</v>
-      </c>
-      <c r="E6" s="11">
-        <v>46174</v>
+        <v>305</v>
+      </c>
+      <c r="D6" s="6">
+        <v>46177</v>
+      </c>
+      <c r="E6" s="6">
+        <v>46177</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>20</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-    </row>
-    <row r="7" spans="1:20" ht="57.6">
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20"/>
+    </row>
+    <row r="7" spans="1:20" ht="43.2">
       <c r="A7" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>226</v>
+        <v>308</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="11">
-        <v>46174</v>
-      </c>
-      <c r="E7" s="11">
-        <v>46174</v>
+        <v>309</v>
+      </c>
+      <c r="D7" s="6">
+        <v>46178</v>
+      </c>
+      <c r="E7" s="6">
+        <v>46178</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" s="5">
-        <v>4.5</v>
+        <v>37</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>312</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J7" s="5"/>
+        <v>310</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
     </row>
     <row r="8" spans="1:20" ht="43.2">
       <c r="A8" s="4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" s="11">
-        <v>46174</v>
-      </c>
-      <c r="E8" s="11">
-        <v>46175</v>
+        <v>306</v>
+      </c>
+      <c r="D8" s="6">
+        <v>46177</v>
+      </c>
+      <c r="E8" s="6">
+        <v>46178</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" s="5">
-        <v>6</v>
+        <v>37</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>307</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>23</v>
+        <v>218</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>24</v>
+        <v>219</v>
       </c>
       <c r="J8" s="5"/>
     </row>
     <row r="9" spans="1:20" ht="43.2">
       <c r="A9" s="4">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" s="11">
+        <v>46178</v>
+      </c>
+      <c r="E9" s="11">
+        <v>46178</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" s="10">
+        <v>4</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="J9" s="5"/>
+    </row>
+    <row r="10" spans="1:20" ht="72">
+      <c r="A10" s="4">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="D10" s="11">
+        <v>46178</v>
+      </c>
+      <c r="E10" s="11">
+        <v>46178</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="J10" s="5"/>
+    </row>
+    <row r="11" spans="1:20" ht="86.4">
+      <c r="A11" s="4"/>
+      <c r="B11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D11" s="11">
+        <v>46178</v>
+      </c>
+      <c r="E11" s="11"/>
+      <c r="F11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="5">
+        <v>6</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" s="5"/>
+    </row>
+    <row r="12" spans="1:20" ht="43.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="5">
+        <v>7</v>
+      </c>
+      <c r="H12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="I12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J12" s="5"/>
+    </row>
+    <row r="13" spans="1:20" ht="57.6">
+      <c r="A13" s="4"/>
+      <c r="B13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="D9" s="11">
-        <v>46174</v>
-      </c>
-      <c r="E9" s="11">
-        <v>46176</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="5">
-        <v>7</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="J9" s="5"/>
-    </row>
-    <row r="10" spans="1:20" ht="57.6">
-      <c r="A10" s="4">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10" s="5">
-        <v>1.3</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:20" ht="57.6">
-      <c r="A11" s="4">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G11" s="5">
-        <v>3</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J11" s="5"/>
-    </row>
-    <row r="12" spans="1:20" ht="43.2">
-      <c r="A12" s="4">
-        <v>11</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:20" ht="86.4">
-      <c r="A13" s="4">
-        <v>12</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>132</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G13" s="5">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>133</v>
+        <v>27</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>134</v>
+        <v>28</v>
       </c>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:20" ht="72">
-      <c r="A14" s="4">
-        <v>13</v>
-      </c>
+    <row r="14" spans="1:20" ht="57.6">
+      <c r="A14" s="4"/>
       <c r="B14" s="5" t="s">
-        <v>135</v>
+        <v>29</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G14" s="5">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>137</v>
+        <v>30</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>138</v>
+        <v>31</v>
       </c>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:20" ht="86.4">
-      <c r="A15" s="4">
-        <v>14</v>
-      </c>
+    <row r="15" spans="1:20" ht="43.2">
+      <c r="A15" s="4"/>
       <c r="B15" s="5" t="s">
-        <v>139</v>
+        <v>32</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" s="5">
-        <v>3.4</v>
+        <v>49</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>141</v>
+        <v>34</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:20" ht="72">
-      <c r="A16" s="4">
-        <v>15</v>
-      </c>
+    <row r="16" spans="1:20" ht="86.4">
+      <c r="A16" s="4"/>
       <c r="B16" s="5" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G16" s="5">
         <v>1</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="J16" s="5"/>
     </row>
     <row r="17" spans="1:10" ht="72">
-      <c r="A17" s="4">
-        <v>16</v>
-      </c>
+      <c r="A17" s="4"/>
       <c r="B17" s="5" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G17" s="5">
+        <v>2.4</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="J17" s="5"/>
+    </row>
+    <row r="18" spans="1:10" ht="86.4">
+      <c r="A18" s="4"/>
+      <c r="B18" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" s="5">
+        <v>3.4</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="J18" s="5"/>
+    </row>
+    <row r="19" spans="1:10" ht="72">
+      <c r="A19" s="4"/>
+      <c r="B19" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G19" s="5">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" spans="1:10" ht="72">
+      <c r="A20" s="4"/>
+      <c r="B20" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="5">
         <v>10</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H20" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="I20" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="I17" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="J17" s="5"/>
+      <c r="J20" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2453,30 +2640,30 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28.8">
       <c r="A1" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" s="9">
         <v>0</v>
@@ -2485,16 +2672,16 @@
         <v>359</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C3" s="9">
         <v>0</v>
@@ -2503,16 +2690,16 @@
         <v>359</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" s="9">
         <v>0</v>
@@ -2521,16 +2708,16 @@
         <v>359</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" s="9">
         <v>0</v>
@@ -2539,34 +2726,34 @@
         <v>330</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="28.8">
       <c r="A6" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" ht="28.8">
       <c r="A7" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C7" s="9">
         <v>0</v>
@@ -2575,16 +2762,16 @@
         <v>359</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" ht="28.8">
       <c r="A8" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C8" s="9">
         <v>0</v>
@@ -2593,16 +2780,16 @@
         <v>359</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" ht="28.8">
       <c r="A9" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C9" s="9">
         <v>1</v>
@@ -2611,34 +2798,34 @@
         <v>0</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="28.8">
       <c r="A10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" s="9">
         <v>0</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>208</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>209</v>
       </c>
       <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C11" s="9">
         <v>1</v>
@@ -2647,34 +2834,34 @@
         <v>0</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>107</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D12" s="5">
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C13" s="9">
         <v>0</v>
@@ -2683,16 +2870,16 @@
         <v>15</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="28.8">
       <c r="A14" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C14" s="9">
         <v>0</v>
@@ -2701,16 +2888,16 @@
         <v>12</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6" ht="28.8">
       <c r="A15" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C15" s="9">
         <v>0</v>
@@ -2719,106 +2906,106 @@
         <v>6</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="28.8">
       <c r="A16" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D16" s="5">
         <v>9</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:6" ht="28.8">
       <c r="A17" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D17" s="5">
         <v>9</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F17" s="5"/>
     </row>
     <row r="18" spans="1:6" ht="28.8">
       <c r="A18" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D18" s="5">
         <v>9</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6" ht="28.8">
       <c r="A19" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D19" s="5">
         <v>8</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6" ht="28.8">
       <c r="A20" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D20" s="5">
         <v>7</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C21" s="9">
         <v>0</v>
@@ -2827,16 +3014,16 @@
         <v>2</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6" ht="28.8">
       <c r="A22" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C22" s="9">
         <v>0</v>
@@ -2845,18 +3032,18 @@
         <v>2</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="28.8">
       <c r="A23" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C23" s="9">
         <v>0</v>
@@ -2865,10 +3052,10 @@
         <v>28</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2894,138 +3081,138 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>55</v>
-      </c>
       <c r="C2" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D2" s="5">
         <v>719</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D3" s="5">
         <v>756</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D4" s="5">
         <v>626</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D5" s="5">
         <v>483</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D6" s="5">
         <v>4</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D7" s="5">
         <v>2</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C8" s="9">
         <v>0</v>
@@ -3034,56 +3221,56 @@
         <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>168</v>
       </c>
       <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="28.8">
       <c r="A10" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C11" s="9">
         <v>0</v>
@@ -3092,16 +3279,16 @@
         <v>4</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C12" s="9">
         <v>0</v>
@@ -3110,34 +3297,34 @@
         <v>9228</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>173</v>
-      </c>
       <c r="E13" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C14" s="9">
         <v>0</v>
@@ -3146,34 +3333,34 @@
         <v>15</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="43.2">
       <c r="A16" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="9">
         <v>0</v>
@@ -3182,18 +3369,18 @@
         <v>27</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C17" s="9">
         <v>0</v>
@@ -3202,88 +3389,88 @@
         <v>5128</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F17" s="5"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D18" s="5">
         <v>4</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D19" s="5">
         <v>20</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D20" s="5">
         <v>361</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>183</v>
       </c>
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C22" s="9">
         <v>0</v>
@@ -3292,88 +3479,88 @@
         <v>9228</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F22" s="5"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D23" s="5">
         <v>15</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F23" s="5"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>79</v>
-      </c>
       <c r="C24" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D24" s="5">
         <v>6616</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F24" s="5"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D25" s="5">
         <v>6441</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F25" s="5"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D26" s="5">
         <v>2</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F26" s="5"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C27" s="9">
         <v>0</v>
@@ -3382,16 +3569,16 @@
         <v>144</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F27" s="5"/>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C28" s="9">
         <v>0</v>
@@ -3400,16 +3587,16 @@
         <v>9228</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F28" s="5"/>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C29" s="9">
         <v>0</v>
@@ -3418,34 +3605,34 @@
         <v>9228</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F29" s="5"/>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>86</v>
-      </c>
       <c r="C30" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D30" s="5">
         <v>6</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F30" s="5"/>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C31" s="9">
         <v>0</v>
@@ -3454,124 +3641,124 @@
         <v>651</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F31" s="5"/>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D32" s="5">
         <v>6</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F32" s="5"/>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D33" s="5">
         <v>3</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F33" s="5"/>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C34" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>192</v>
-      </c>
       <c r="E34" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F34" s="5"/>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C35" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>194</v>
-      </c>
       <c r="E35" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F35" s="5"/>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>93</v>
-      </c>
       <c r="C36" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>195</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>196</v>
       </c>
       <c r="F36" s="5"/>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E37" s="5" t="s">
         <v>195</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>196</v>
       </c>
       <c r="F37" s="5"/>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C38" s="9">
         <v>1</v>
@@ -3580,16 +3767,16 @@
         <v>0</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F38" s="5"/>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C39" s="9">
         <v>0</v>
@@ -3598,25 +3785,25 @@
         <v>1</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F39" s="5"/>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D40" s="5">
         <v>1</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F40" s="5"/>
     </row>
@@ -3959,95 +4146,95 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>230</v>
-      </c>
       <c r="C34" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>252</v>
-      </c>
       <c r="E35" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E36" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="B37" s="5" t="s">
-        <v>233</v>
-      </c>
       <c r="C37" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>235</v>
-      </c>
       <c r="C38" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B39" s="5" t="s">
-        <v>238</v>
-      </c>
       <c r="C39" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -4060,103 +4247,103 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B46" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>252</v>
-      </c>
       <c r="E46" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E47" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>238</v>
-      </c>
       <c r="C51" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -4166,7 +4353,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
@@ -4183,43 +4370,43 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C57" s="5"/>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B58" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>233</v>
       </c>
       <c r="C58" s="5"/>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B60" s="5" t="s">
         <v>259</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>260</v>
       </c>
       <c r="C60" s="4"/>
     </row>
@@ -4235,35 +4422,35 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C64" s="5"/>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C65" s="5"/>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C66" s="5"/>
     </row>
@@ -4410,7 +4597,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0706F5C-AC4A-42FB-8855-D5F3F3D2DC4D}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="8" customWidth="1"/>
@@ -4424,22 +4611,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.8">
@@ -4447,13 +4634,13 @@
         <v>46170</v>
       </c>
       <c r="B2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>53</v>
       </c>
       <c r="F2" s="7">
         <v>46171</v>
@@ -4464,16 +4651,16 @@
         <v>46170</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>49</v>
       </c>
       <c r="F3" s="7">
         <v>46171</v>
@@ -4484,13 +4671,13 @@
         <v>46170</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>263</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>264</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="7">
@@ -4502,13 +4689,13 @@
         <v>46175</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>279</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>280</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="7">
@@ -4520,13 +4707,13 @@
         <v>46175</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>282</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="7">
@@ -4538,13 +4725,13 @@
         <v>46176</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>285</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>286</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="7">
@@ -4556,13 +4743,13 @@
         <v>46176</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="7">
@@ -4574,18 +4761,36 @@
         <v>46176</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>288</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>289</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="7">
         <v>46176</v>
       </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="7">
+        <v>46176</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="F10" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4602,47 +4807,47 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="16" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="16" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="16" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="16" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="1:1">
@@ -4650,50 +4855,558 @@
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="16" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="16" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="16" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="16" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E42101E-BA60-49BD-B385-DC06AE7D6FD6}">
+  <dimension ref="A1:T17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.88671875" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5546875" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="57.6">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="6">
+        <v>46170</v>
+      </c>
+      <c r="E2" s="6">
+        <v>46174</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="J2" s="5"/>
+    </row>
+    <row r="3" spans="1:20" ht="43.2">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D3" s="6">
+        <v>46170</v>
+      </c>
+      <c r="E3" s="6">
+        <v>46174</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+    </row>
+    <row r="4" spans="1:20" ht="57.6">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="6">
+        <v>46174</v>
+      </c>
+      <c r="E4" s="6">
+        <v>46174</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="5">
+        <v>2</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="J4" s="5"/>
+    </row>
+    <row r="5" spans="1:20" ht="28.8">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="D5" s="11">
+        <v>46174</v>
+      </c>
+      <c r="E5" s="11">
+        <v>46174</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="10">
+        <v>3</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="I5" s="10"/>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" spans="1:20" ht="43.2">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D6" s="11">
+        <v>46174</v>
+      </c>
+      <c r="E6" s="11">
+        <v>46174</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" spans="1:20" ht="57.6">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="11">
+        <v>46174</v>
+      </c>
+      <c r="E7" s="11">
+        <v>46174</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8" spans="1:20" ht="43.2">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="11">
+        <v>46174</v>
+      </c>
+      <c r="E8" s="11">
+        <v>46175</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="5">
+        <v>6</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9" spans="1:20" ht="43.2">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="11">
+        <v>46174</v>
+      </c>
+      <c r="E9" s="11">
+        <v>46176</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="5">
+        <v>7</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J9" s="5"/>
+    </row>
+    <row r="10" spans="1:20" ht="57.6">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" s="5"/>
+    </row>
+    <row r="11" spans="1:20" ht="57.6">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="5">
+        <v>3</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J11" s="5"/>
+    </row>
+    <row r="12" spans="1:20" ht="43.2">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="J12" s="5"/>
+    </row>
+    <row r="13" spans="1:20" ht="86.4">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="5">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="J13" s="5"/>
+    </row>
+    <row r="14" spans="1:20" ht="72">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="5">
+        <v>2.4</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="J14" s="5"/>
+    </row>
+    <row r="15" spans="1:20" ht="86.4">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="5">
+        <v>3.4</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="J15" s="5"/>
+    </row>
+    <row r="16" spans="1:20" ht="72">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" s="5">
+        <v>1</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" spans="1:10" ht="72">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="5">
+        <v>10</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="J17" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
New silver loader and cleanup of files/folders
</commit_message>
<xml_diff>
--- a/Projektplan.xlsx
+++ b/Projektplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michael.brostrom\Documents\GitHub\statistik-freshdesk-linear\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8584E54-1A62-41CB-A4A9-EB8198036C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9056305-F46A-4A8F-875F-4065CBD8C1E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-46188" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{6423C684-42E7-44D6-BC0D-A51FB6EB8C31}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="321">
   <si>
     <t>Steg 2</t>
   </si>
@@ -1097,9 +1097,6 @@
     <t xml:space="preserve">SQL Server Authentication-login i /credentials </t>
   </si>
   <si>
-    <t>Städat bort mycket irrelevant från Freshdesk och en del från Linear.</t>
-  </si>
-  <si>
     <t>Generera DimDate för 2025–2035 med daglig granularitet och diverse "smarta" kolumner för hanteringen.</t>
   </si>
   <si>
@@ -1107,6 +1104,34 @@
   </si>
   <si>
     <t>Skapa vyer i Gold-lagret så att PBI via dessa kommer åt data från Silverlagret (som blir det sista som uppdateras från rådata - via bronze).</t>
+  </si>
+  <si>
+    <t>Guldlagret</t>
+  </si>
+  <si>
+    <t>Tillagd funktionalitet för enklare visualisering</t>
+  </si>
+  <si>
+    <t>Görs automatiskt via Python-script</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Städat bort mycket irrelevant från Freshdesk och en del från Linear. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Automatisering för hämtning av bronsdata.</t>
+    </r>
+  </si>
+  <si>
+    <t>Power BI</t>
   </si>
 </sst>
 </file>
@@ -1178,12 +1203,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1210,7 +1241,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1262,6 +1293,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1625,10 +1659,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}" name="Table3" displayName="Table3" ref="A3:J20" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
-  <autoFilter ref="A3:J20" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:J20">
-    <sortCondition ref="A4:A20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}" name="Table3" displayName="Table3" ref="A3:J21" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+  <autoFilter ref="A3:J21" xr:uid="{439807E8-31AA-4E2E-81B8-9D708AC63526}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:J21">
+    <sortCondition ref="A4:A21"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{621EA786-D68B-4811-8816-275E67518CF7}" name="ID" dataDxfId="32"/>
@@ -2099,7 +2133,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4FCEBCE-FCD7-407D-A82B-012E341489A8}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
@@ -2315,11 +2349,11 @@
         <v>218</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>219</v>
+        <v>318</v>
       </c>
       <c r="J8" s="5"/>
     </row>
-    <row r="9" spans="1:20" ht="43.2">
+    <row r="9" spans="1:20" ht="57.6">
       <c r="A9" s="4">
         <v>5</v>
       </c>
@@ -2332,11 +2366,9 @@
       <c r="D9" s="11">
         <v>46178</v>
       </c>
-      <c r="E9" s="11">
-        <v>46178</v>
-      </c>
+      <c r="E9" s="11"/>
       <c r="F9" s="5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G9" s="10">
         <v>4</v>
@@ -2344,8 +2376,8 @@
       <c r="H9" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>313</v>
+      <c r="I9" s="21" t="s">
+        <v>319</v>
       </c>
       <c r="J9" s="5"/>
     </row>
@@ -2357,7 +2389,7 @@
         <v>18</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D10" s="11">
         <v>46178</v>
@@ -2373,163 +2405,133 @@
         <v>42</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J10" s="5"/>
     </row>
     <row r="11" spans="1:20" ht="86.4">
-      <c r="A11" s="4"/>
+      <c r="A11" s="4">
+        <v>7</v>
+      </c>
       <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D11" s="11">
         <v>46178</v>
       </c>
-      <c r="E11" s="11"/>
+      <c r="E11" s="11">
+        <v>46178</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="G11" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>22</v>
+        <v>316</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>23</v>
+        <v>317</v>
       </c>
       <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="1:20" ht="43.2">
+    <row r="12" spans="1:20">
       <c r="A12" s="4"/>
-      <c r="B12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>125</v>
-      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
       <c r="D12" s="11"/>
       <c r="E12" s="11"/>
-      <c r="F12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" s="5">
-        <v>7</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>40</v>
-      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
       <c r="J12" s="5"/>
     </row>
-    <row r="13" spans="1:20" ht="57.6">
+    <row r="13" spans="1:20" ht="43.2">
       <c r="A13" s="4"/>
       <c r="B13" s="5" t="s">
-        <v>26</v>
+        <v>320</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+        <v>125</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="5">
-        <v>1.3</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:20" ht="57.6">
+    <row r="14" spans="1:20">
       <c r="A14" s="4"/>
-      <c r="B14" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>127</v>
-      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
-      <c r="F14" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G14" s="5">
-        <v>3</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:20" ht="43.2">
+    <row r="15" spans="1:20" ht="57.6">
       <c r="A15" s="4"/>
       <c r="B15" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>33</v>
-      </c>
+      <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>129</v>
+        <v>31</v>
       </c>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:20" ht="86.4">
+    <row r="16" spans="1:20" ht="43.2">
       <c r="A16" s="4"/>
       <c r="B16" s="5" t="s">
-        <v>130</v>
+        <v>32</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="5">
-        <v>1</v>
-      </c>
+      <c r="G16" s="5"/>
       <c r="H16" s="5" t="s">
-        <v>132</v>
+        <v>34</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="1:10" ht="72">
+    <row r="17" spans="1:10" ht="86.4">
       <c r="A17" s="4"/>
       <c r="B17" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
@@ -2537,47 +2539,35 @@
         <v>49</v>
       </c>
       <c r="G17" s="5">
-        <v>2.4</v>
+        <v>1</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" spans="1:10" ht="86.4">
+    <row r="18" spans="1:10">
       <c r="A18" s="4"/>
-      <c r="B18" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>139</v>
-      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
-      <c r="F18" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" s="5">
-        <v>3.4</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>141</v>
-      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
       <c r="J18" s="5"/>
     </row>
-    <row r="19" spans="1:10" ht="72">
+    <row r="19" spans="1:10" ht="86.4">
       <c r="A19" s="4"/>
       <c r="B19" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
@@ -2585,39 +2575,51 @@
         <v>49</v>
       </c>
       <c r="G19" s="5">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="J19" s="5"/>
     </row>
-    <row r="20" spans="1:10" ht="72">
+    <row r="20" spans="1:10">
       <c r="A20" s="4"/>
-      <c r="B20" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>147</v>
-      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="1:10" ht="72">
+      <c r="A21" s="4"/>
+      <c r="B21" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G21" s="5">
         <v>10</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H21" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="I20" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="J20" s="5"/>
+      <c r="J21" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>